<commit_message>
Latest code for Czechia, Its working
</commit_message>
<xml_diff>
--- a/Data/testDataCzechia - Copy - Copy.xlsx
+++ b/Data/testDataCzechia - Copy - Copy.xlsx
@@ -1,15 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{18986918-1B52-4299-8CB4-4796075B3B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176"/>
+    <workbookView xWindow="20" yWindow="620" windowWidth="19180" windowHeight="10180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -601,77 +616,77 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="14"/>
       <color rgb="FFFF0000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <family val="2"/>
-      <scheme val="minor"/>
       <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <color rgb="FF000000"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -690,7 +705,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -708,7 +723,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.3999755851924192"/>
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -725,13 +740,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.0499893185216834"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -760,9 +775,15 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -772,8 +793,12 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -807,10 +832,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1300,14 +1333,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CX7"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="102" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:102" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1615,7 +1648,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" ht="19.2" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:102" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>92</v>
       </c>
@@ -1721,9 +1754,9 @@
       <c r="AJ2" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="AK2" s="28">
+      <c r="AK2" s="28" t="str">
         <f t="shared" ref="AK2:AK7" si="1">AH2</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AL2" s="29">
         <f t="shared" ref="AL2:AL7" si="2">K2</f>
@@ -1925,7 +1958,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="3" ht="19.2" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:102" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>143</v>
       </c>
@@ -2031,9 +2064,9 @@
       <c r="AJ3" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="AK3" s="28">
+      <c r="AK3" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AL3" s="29">
         <f t="shared" si="2"/>
@@ -2235,7 +2268,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="4" ht="19.2" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:102" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>154</v>
       </c>
@@ -2327,8 +2360,8 @@
         <v>20</v>
       </c>
       <c r="AH4" s="26">
-        <f>TODAY()+365</f>
-        <v>45953</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46031</v>
       </c>
       <c r="AI4" s="27" t="s">
         <v>114</v>
@@ -2337,8 +2370,8 @@
         <v>115</v>
       </c>
       <c r="AK4" s="28">
-        <f t="shared" si="1"/>
-        <v>45953</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46031</v>
       </c>
       <c r="AL4" s="29">
         <f t="shared" si="2"/>
@@ -2540,7 +2573,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="5" ht="19.2" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:102" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>165</v>
       </c>
@@ -2632,8 +2665,8 @@
         <v>40</v>
       </c>
       <c r="AH5" s="26">
-        <f>TODAY()+365</f>
-        <v>45953</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46031</v>
       </c>
       <c r="AI5" s="27" t="s">
         <v>114</v>
@@ -2642,8 +2675,8 @@
         <v>115</v>
       </c>
       <c r="AK5" s="28">
-        <f t="shared" si="1"/>
-        <v>45953</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46031</v>
       </c>
       <c r="AL5" s="29">
         <f t="shared" si="2"/>
@@ -2845,7 +2878,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="6" ht="19.2" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:102" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>174</v>
       </c>
@@ -2937,8 +2970,8 @@
         <v>16</v>
       </c>
       <c r="AH6" s="26">
-        <f>TODAY()+365</f>
-        <v>45953</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46031</v>
       </c>
       <c r="AI6" s="27" t="s">
         <v>179</v>
@@ -2947,8 +2980,8 @@
         <v>115</v>
       </c>
       <c r="AK6" s="28">
-        <f t="shared" si="1"/>
-        <v>45953</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>46031</v>
       </c>
       <c r="AL6" s="29">
         <f t="shared" si="2"/>
@@ -3150,7 +3183,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" ht="19.2" customHeight="1" spans="1:102" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:102" ht="19.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>184</v>
       </c>
@@ -3250,9 +3283,9 @@
       <c r="AJ7" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="AK7" s="28">
+      <c r="AK7" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AL7" s="29">
         <f t="shared" si="2"/>
@@ -3455,29 +3488,17 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ7">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ7 Y2:Y7 W2:W7 T2:T7" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($E1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2:BR7">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2:BR7 J2:J7" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J7">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T7">
-      <formula1>INDIRECT($E1)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W7">
-      <formula1>INDIRECT($E1)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y7">
-      <formula1>INDIRECT($E1)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="V2" r:id="rId1"/>
-    <hyperlink ref="V3" r:id="rId2"/>
+    <hyperlink ref="V2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="V3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>